<commit_message>
feat: cosme-ranking-products scraper + deprecate cosme + word_clinical updates
- Rename bd_scrapers/cosme → cosme_deprecated y gli_scrapers/cosme → cosme_deprecated (scraper original reemplazado)
- Agregar bd_scrapers/cosme-ranking-products v1 (sc_browser + sc_code) con dom_map, results y registry
- Agregar gli_scrapers/cosme_ranking_products: middleware Python (client, models, config, tool_schema, tests)
- Agregar docs/fase3/cosme-ranking-products-handoff.md y actualizar docs/specs/scrapers/cosme.md
- Agregar .agents/skills/snowflake-json-load (skill de carga emergencia JSON → Snowflake)
- word_clinical: formula_parser.py nuevo, ajustes en models/pdf_extractor/runner
- Actualizar docs/ddl/DEV_STG_GNM_MEX.sql y catálogo xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/specs/brightd-scrapers/listado de scrapers.xlsx
+++ b/docs/specs/brightd-scrapers/listado de scrapers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Genomma Lab\OneDrive\Genomma\MicroDockerTests\brightdata-scrapers\docs\specs\brightd-scrapers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2543FB4-906E-453A-8BCA-326E788678AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE818B8D-2969-4051-8773-96F10C48D06F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{7CB1BBF7-238F-41B5-9831-A0BD931B9AB4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7CB1BBF7-238F-41B5-9831-A0BD931B9AB4}"/>
   </bookViews>
   <sheets>
     <sheet name="scrapers" sheetId="3" r:id="rId1"/>
@@ -1194,7 +1194,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" tooltip="https://marcia.impi.gob.mx/marcas/search/quick" xr:uid="{17ED3423-1A9B-4292-B719-B130EF359577}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{17ED3423-1A9B-4292-B719-B130EF359577}"/>
     <hyperlink ref="D3" r:id="rId2" tooltip="https://www.sic.gov.co/marcas" xr:uid="{B75BAC3F-E308-40B1-94A5-9892E888CEB8}"/>
     <hyperlink ref="D4" r:id="rId3" tooltip="https://www.uspto.gov/trademarks/search" xr:uid="{A475F351-19FF-4F91-82D4-C7BAC65549D5}"/>
     <hyperlink ref="D5" r:id="rId4" tooltip="https://portaltramites.inpi.gob.ar/marcasconsultas/busqueda" xr:uid="{D46CA269-07FA-497D-BADD-28C0CFF1E8A2}"/>

</xml_diff>